<commit_message>
low quality data need to be removed
</commit_message>
<xml_diff>
--- a/noodlepy/data/Biofluid_list_annotated_v4.xlsx
+++ b/noodlepy/data/Biofluid_list_annotated_v4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifeigu/Documents/Carney_Lab/NoodlePy/noodlepy/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED8611D-07BC-D248-BCB5-4BE474D4C10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB4CA3F-329E-6A4B-B3D8-B3C99C2F63AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34080" yWindow="500" windowWidth="30240" windowHeight="18880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -195,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -212,15 +212,31 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,21 +554,23 @@
   <dimension ref="A1:S219"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" style="10" customWidth="1"/>
     <col min="2" max="2" width="12.5" style="2" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="12" style="2" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="0" style="2" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="11" style="2"/>
-    <col min="6" max="6" width="27.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11" style="10"/>
+    <col min="6" max="6" width="27.83203125" style="15" customWidth="1"/>
     <col min="7" max="7" width="11" style="2"/>
     <col min="8" max="8" width="18.5" style="2" customWidth="1"/>
-    <col min="9" max="14" width="11" style="2"/>
+    <col min="9" max="9" width="11" style="2"/>
+    <col min="10" max="11" width="0" style="2" hidden="1" customWidth="1"/>
+    <col min="12" max="14" width="11" style="2"/>
     <col min="15" max="15" width="11" style="3"/>
     <col min="16" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -564,10 +582,10 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="14" t="s">
         <v>20</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -576,18 +594,18 @@
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="16" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
+      <c r="A2" s="10">
         <v>166</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H2" s="2">
@@ -604,13 +622,13 @@
       <c r="S2" s="4"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="7">
+      <c r="A3" s="10">
         <v>191</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H3" s="2">
@@ -627,7 +645,7 @@
       <c r="S3" s="4"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+      <c r="A4" s="10">
         <v>272</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -639,10 +657,10 @@
       <c r="D4" s="2">
         <v>73</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="E4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="2">
@@ -666,7 +684,7 @@
       <c r="S4" s="4"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="A5" s="10">
         <v>275</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -678,10 +696,10 @@
       <c r="D5" s="2">
         <v>86</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="E5" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="2">
@@ -705,7 +723,7 @@
       <c r="S5" s="4"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="A6" s="10">
         <v>276</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -717,10 +735,10 @@
       <c r="D6" s="2">
         <v>63</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="2">
@@ -744,7 +762,7 @@
       <c r="S6" s="4"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="A7" s="10">
         <v>277</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -756,10 +774,10 @@
       <c r="D7" s="2">
         <v>30</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="2" t="s">
+      <c r="E7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="2">
@@ -783,7 +801,7 @@
       <c r="S7" s="4"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="A8" s="10">
         <v>278</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -795,10 +813,10 @@
       <c r="D8" s="2">
         <v>27</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="2">
@@ -822,7 +840,7 @@
       <c r="S8" s="4"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+      <c r="A9" s="10">
         <v>279</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -834,10 +852,10 @@
       <c r="D9" s="2">
         <v>29</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="E9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="2">
@@ -857,7 +875,7 @@
       <c r="S9" s="4"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="A10" s="10">
         <v>280</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -869,10 +887,10 @@
       <c r="D10" s="2">
         <v>66</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="E10" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G10" s="2">
@@ -892,7 +910,7 @@
       <c r="S10" s="4"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+      <c r="A11" s="10">
         <v>281</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -904,10 +922,10 @@
       <c r="D11" s="2">
         <v>43</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="E11" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>12</v>
       </c>
       <c r="G11" s="2">
@@ -927,7 +945,7 @@
       <c r="S11" s="4"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+      <c r="A12" s="10">
         <v>284</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -939,10 +957,10 @@
       <c r="D12" s="2">
         <v>53</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="E12" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="15" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="2">
@@ -962,7 +980,7 @@
       <c r="S12" s="4"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+      <c r="A13" s="10">
         <v>286</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -974,10 +992,10 @@
       <c r="D13" s="2">
         <v>63</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="E13" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G13" s="2">
@@ -997,7 +1015,7 @@
       <c r="S13" s="4"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+      <c r="A14" s="10">
         <v>287</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -1009,10 +1027,10 @@
       <c r="D14" s="2">
         <v>72</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="E14" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="2">
@@ -1032,7 +1050,7 @@
       <c r="S14" s="4"/>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+      <c r="A15" s="10">
         <v>288</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -1044,10 +1062,10 @@
       <c r="D15" s="2">
         <v>31</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G15" s="2" t="s">
@@ -1067,7 +1085,7 @@
       <c r="S15" s="4"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+      <c r="A16" s="10">
         <v>289</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -1079,10 +1097,10 @@
       <c r="D16" s="2">
         <v>74</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G16" s="2">
@@ -1102,7 +1120,7 @@
       <c r="S16" s="4"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+      <c r="A17" s="10">
         <v>291</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -1114,10 +1132,10 @@
       <c r="D17" s="2">
         <v>72</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="E17" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="2">
@@ -1137,7 +1155,7 @@
       <c r="S17" s="4"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="A18" s="10">
         <v>292</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -1149,10 +1167,10 @@
       <c r="D18" s="2">
         <v>51</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="E18" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G18" s="2">
@@ -1172,7 +1190,7 @@
       <c r="S18" s="4"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="A19" s="10">
         <v>293</v>
       </c>
       <c r="B19" s="2" t="s">
@@ -1184,10 +1202,10 @@
       <c r="D19" s="2">
         <v>50</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" s="2" t="s">
+      <c r="E19" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G19" s="2">
@@ -1207,7 +1225,7 @@
       <c r="S19" s="4"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="A20" s="10">
         <v>294</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -1219,10 +1237,10 @@
       <c r="D20" s="2">
         <v>44</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="15" t="s">
         <v>16</v>
       </c>
       <c r="G20" s="2">
@@ -1242,7 +1260,7 @@
       <c r="S20" s="4"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+      <c r="A21" s="10">
         <v>295</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -1254,10 +1272,10 @@
       <c r="D21" s="2">
         <v>71</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G21" s="2">
@@ -1277,7 +1295,7 @@
       <c r="S21" s="4"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+      <c r="A22" s="10">
         <v>296</v>
       </c>
       <c r="B22" s="2" t="s">
@@ -1289,10 +1307,10 @@
       <c r="D22" s="2">
         <v>66</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" s="2" t="s">
+      <c r="E22" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G22" s="2">
@@ -1312,7 +1330,7 @@
       <c r="S22" s="4"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+      <c r="A23" s="10">
         <v>297</v>
       </c>
       <c r="B23" s="2" t="s">
@@ -1324,10 +1342,10 @@
       <c r="D23" s="2">
         <v>77</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23" s="2" t="s">
+      <c r="E23" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G23" s="2">
@@ -1347,7 +1365,7 @@
       <c r="S23" s="4"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+      <c r="A24" s="10">
         <v>298</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -1359,10 +1377,10 @@
       <c r="D24" s="2">
         <v>81</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F24" s="2" t="s">
+      <c r="E24" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F24" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G24" s="2">
@@ -1382,7 +1400,7 @@
       <c r="S24" s="4"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+      <c r="A25" s="10">
         <v>299</v>
       </c>
       <c r="B25" s="2" t="s">
@@ -1391,10 +1409,10 @@
       <c r="D25" s="2">
         <v>76</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G25" s="2">
@@ -1414,7 +1432,7 @@
       <c r="S25" s="4"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+      <c r="A26" s="10">
         <v>300</v>
       </c>
       <c r="B26" s="2" t="s">
@@ -1426,10 +1444,10 @@
       <c r="D26" s="2">
         <v>79</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" s="2" t="s">
+      <c r="E26" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G26" s="2">
@@ -1449,7 +1467,7 @@
       <c r="S26" s="4"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+      <c r="A27" s="10">
         <v>301</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -1461,10 +1479,10 @@
       <c r="D27" s="2">
         <v>57</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F27" s="2" t="s">
+      <c r="E27" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" s="15" t="s">
         <v>12</v>
       </c>
       <c r="G27" s="2">
@@ -1484,7 +1502,7 @@
       <c r="S27" s="4"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+      <c r="A28" s="10">
         <v>302</v>
       </c>
       <c r="B28" s="2" t="s">
@@ -1496,10 +1514,10 @@
       <c r="D28" s="2">
         <v>70</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="2">
@@ -1519,7 +1537,7 @@
       <c r="S28" s="4"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+      <c r="A29" s="10">
         <v>304</v>
       </c>
       <c r="B29" s="2" t="s">
@@ -1531,10 +1549,10 @@
       <c r="D29" s="2">
         <v>67</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F29" s="2" t="s">
+      <c r="E29" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G29" s="2">
@@ -1554,7 +1572,7 @@
       <c r="S29" s="4"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+      <c r="A30" s="10">
         <v>305</v>
       </c>
       <c r="B30" s="2" t="s">
@@ -1566,10 +1584,10 @@
       <c r="D30" s="2">
         <v>58</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F30" s="2" t="s">
+      <c r="E30" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F30" s="15" t="s">
         <v>18</v>
       </c>
       <c r="G30" s="2">
@@ -1589,7 +1607,7 @@
       <c r="S30" s="4"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+      <c r="A31" s="10">
         <v>306</v>
       </c>
       <c r="B31" s="2" t="s">
@@ -1601,10 +1619,10 @@
       <c r="D31" s="2">
         <v>56</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F31" s="2" t="s">
+      <c r="E31" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F31" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G31" s="2">
@@ -1624,7 +1642,7 @@
       <c r="S31" s="4"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+      <c r="A32" s="10">
         <v>309</v>
       </c>
       <c r="B32" s="2" t="s">
@@ -1633,10 +1651,10 @@
       <c r="D32" s="2">
         <v>61</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F32" s="2" t="s">
+      <c r="E32" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F32" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G32" s="2">
@@ -1656,7 +1674,7 @@
       <c r="S32" s="4"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+      <c r="A33" s="10">
         <v>310</v>
       </c>
       <c r="B33" s="2" t="s">
@@ -1668,10 +1686,10 @@
       <c r="D33" s="2">
         <v>65</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F33" s="2" t="s">
+      <c r="E33" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F33" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G33" s="2">
@@ -1691,7 +1709,7 @@
       <c r="S33" s="4"/>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+      <c r="A34" s="10">
         <v>312</v>
       </c>
       <c r="B34" s="2" t="s">
@@ -1703,10 +1721,10 @@
       <c r="D34" s="2">
         <v>63</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F34" s="2" t="s">
+      <c r="E34" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F34" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G34" s="2">
@@ -1726,7 +1744,7 @@
       <c r="S34" s="4"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+      <c r="A35" s="10">
         <v>313</v>
       </c>
       <c r="B35" s="2" t="s">
@@ -1738,10 +1756,10 @@
       <c r="D35" s="2">
         <v>64</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F35" s="2" t="s">
+      <c r="E35" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G35" s="2">
@@ -1761,7 +1779,7 @@
       <c r="S35" s="4"/>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+      <c r="A36" s="10">
         <v>314</v>
       </c>
       <c r="B36" s="2" t="s">
@@ -1773,10 +1791,10 @@
       <c r="D36" s="2">
         <v>57</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F36" s="2" t="s">
+      <c r="E36" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F36" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G36" s="2">
@@ -1796,7 +1814,7 @@
       <c r="S36" s="4"/>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+      <c r="A37" s="10">
         <v>315</v>
       </c>
       <c r="B37" s="2" t="s">
@@ -1808,10 +1826,10 @@
       <c r="D37" s="2">
         <v>72</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F37" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G37" s="2">
@@ -1831,7 +1849,7 @@
       <c r="S37" s="4"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+      <c r="A38" s="10">
         <v>316</v>
       </c>
       <c r="B38" s="2" t="s">
@@ -1843,10 +1861,10 @@
       <c r="D38" s="2">
         <v>65</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F38" s="2" t="s">
+      <c r="E38" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F38" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G38" s="2">
@@ -1866,7 +1884,7 @@
       <c r="S38" s="4"/>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+      <c r="A39" s="10">
         <v>317</v>
       </c>
       <c r="C39" s="2" t="s">
@@ -1875,10 +1893,10 @@
       <c r="D39" s="2">
         <v>79</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F39" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G39" s="2">
@@ -1898,7 +1916,7 @@
       <c r="S39" s="4"/>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+      <c r="A40" s="10">
         <v>318</v>
       </c>
       <c r="B40" s="2" t="s">
@@ -1910,10 +1928,10 @@
       <c r="D40" s="2">
         <v>78</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F40" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G40" s="2">
@@ -1933,7 +1951,7 @@
       <c r="S40" s="4"/>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+      <c r="A41" s="10">
         <v>319</v>
       </c>
       <c r="B41" s="2" t="s">
@@ -1945,10 +1963,10 @@
       <c r="D41" s="2">
         <v>62</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F41" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G41" s="2">
@@ -1968,7 +1986,7 @@
       <c r="S41" s="4"/>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+      <c r="A42" s="10">
         <v>320</v>
       </c>
       <c r="B42" s="2" t="s">
@@ -1980,10 +1998,10 @@
       <c r="D42" s="2">
         <v>54</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42" s="2" t="s">
+      <c r="E42" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G42" s="2">
@@ -2003,7 +2021,7 @@
       <c r="S42" s="4"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+      <c r="A43" s="10">
         <v>321</v>
       </c>
       <c r="B43" s="2" t="s">
@@ -2015,10 +2033,10 @@
       <c r="D43" s="2">
         <v>47</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="F43" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G43" s="2">
@@ -2038,7 +2056,7 @@
       <c r="S43" s="4"/>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+      <c r="A44" s="10">
         <v>322</v>
       </c>
       <c r="B44" s="2" t="s">
@@ -2050,10 +2068,10 @@
       <c r="D44" s="2">
         <v>69</v>
       </c>
-      <c r="E44" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F44" s="2" t="s">
+      <c r="E44" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G44" s="2">
@@ -2073,7 +2091,7 @@
       <c r="S44" s="4"/>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+      <c r="A45" s="10">
         <v>323</v>
       </c>
       <c r="B45" s="2" t="s">
@@ -2082,10 +2100,10 @@
       <c r="D45" s="2">
         <v>78</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F45" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G45" s="2">
@@ -2105,7 +2123,7 @@
       <c r="S45" s="4"/>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+      <c r="A46" s="10">
         <v>324</v>
       </c>
       <c r="B46" s="2" t="s">
@@ -2117,10 +2135,10 @@
       <c r="D46" s="2">
         <v>57</v>
       </c>
-      <c r="E46" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F46" s="2" t="s">
+      <c r="E46" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G46" s="2">
@@ -2140,7 +2158,7 @@
       <c r="S46" s="4"/>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+      <c r="A47" s="10">
         <v>325</v>
       </c>
       <c r="B47" s="2" t="s">
@@ -2149,10 +2167,10 @@
       <c r="D47" s="2">
         <v>78</v>
       </c>
-      <c r="E47" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F47" s="2" t="s">
+      <c r="E47" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F47" s="15" t="s">
         <v>13</v>
       </c>
       <c r="G47" s="2">
@@ -2172,7 +2190,7 @@
       <c r="S47" s="4"/>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+      <c r="A48" s="10">
         <v>326</v>
       </c>
       <c r="B48" s="2" t="s">
@@ -2184,10 +2202,10 @@
       <c r="D48" s="2">
         <v>58</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="E48" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G48" s="2">
@@ -2207,7 +2225,7 @@
       <c r="S48" s="4"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+      <c r="A49" s="10">
         <v>327</v>
       </c>
       <c r="B49" s="2" t="s">
@@ -2219,10 +2237,10 @@
       <c r="D49" s="2">
         <v>61</v>
       </c>
-      <c r="E49" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F49" s="2" t="s">
+      <c r="E49" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F49" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G49" s="2">
@@ -2242,7 +2260,7 @@
       <c r="S49" s="4"/>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+      <c r="A50" s="10">
         <v>328</v>
       </c>
       <c r="B50" s="2" t="s">
@@ -2251,10 +2269,10 @@
       <c r="D50" s="2">
         <v>71</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G50" s="2">
@@ -2274,7 +2292,7 @@
       <c r="S50" s="4"/>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+      <c r="A51" s="10">
         <v>329</v>
       </c>
       <c r="B51" s="2" t="s">
@@ -2286,10 +2304,10 @@
       <c r="D51" s="2">
         <v>72</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F51" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="2">
@@ -2309,7 +2327,7 @@
       <c r="S51" s="4"/>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
+      <c r="A52" s="10">
         <v>330</v>
       </c>
       <c r="B52" s="2" t="s">
@@ -2321,10 +2339,10 @@
       <c r="D52" s="2">
         <v>30</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="E52" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="F52" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G52" s="2">
@@ -2344,7 +2362,7 @@
       <c r="S52" s="4"/>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+      <c r="A53" s="10">
         <v>331</v>
       </c>
       <c r="B53" s="2" t="s">
@@ -2356,10 +2374,10 @@
       <c r="D53" s="2">
         <v>76</v>
       </c>
-      <c r="E53" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F53" s="2" t="s">
+      <c r="E53" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F53" s="15" t="s">
         <v>12</v>
       </c>
       <c r="G53" s="2">
@@ -2379,7 +2397,7 @@
       <c r="S53" s="4"/>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
+      <c r="A54" s="10">
         <v>334</v>
       </c>
       <c r="B54" s="2" t="s">
@@ -2391,10 +2409,10 @@
       <c r="D54" s="2">
         <v>67</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F54" s="2" t="s">
+      <c r="E54" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F54" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G54" s="2">
@@ -2414,7 +2432,7 @@
       <c r="S54" s="4"/>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+      <c r="A55" s="10">
         <v>335</v>
       </c>
       <c r="B55" s="2" t="s">
@@ -2423,10 +2441,10 @@
       <c r="D55" s="2">
         <v>76</v>
       </c>
-      <c r="E55" s="2" t="s">
+      <c r="E55" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="F55" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G55" s="2">
@@ -2446,7 +2464,7 @@
       <c r="S55" s="4"/>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+      <c r="A56" s="10">
         <v>336</v>
       </c>
       <c r="B56" s="2" t="s">
@@ -2458,10 +2476,10 @@
       <c r="D56" s="2">
         <v>66</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="E56" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F56" s="2" t="s">
+      <c r="F56" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G56" s="2">
@@ -2481,7 +2499,7 @@
       <c r="S56" s="4"/>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+      <c r="A57" s="10">
         <v>337</v>
       </c>
       <c r="B57" s="2" t="s">
@@ -2493,10 +2511,10 @@
       <c r="D57" s="2">
         <v>58</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E57" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F57" s="2" t="s">
+      <c r="F57" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G57" s="2">
@@ -2516,7 +2534,7 @@
       <c r="S57" s="4"/>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+      <c r="A58" s="10">
         <v>338</v>
       </c>
       <c r="C58" s="2" t="s">
@@ -2525,10 +2543,10 @@
       <c r="D58" s="2">
         <v>60</v>
       </c>
-      <c r="E58" s="2" t="s">
+      <c r="E58" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="F58" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G58" s="2">
@@ -2548,7 +2566,7 @@
       <c r="S58" s="4"/>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
+      <c r="A59" s="10">
         <v>339</v>
       </c>
       <c r="B59" s="2" t="s">
@@ -2560,10 +2578,10 @@
       <c r="D59" s="2">
         <v>65</v>
       </c>
-      <c r="E59" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F59" s="2" t="s">
+      <c r="E59" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G59" s="2">
@@ -2583,7 +2601,7 @@
       <c r="S59" s="4"/>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
+      <c r="A60" s="10">
         <v>340</v>
       </c>
       <c r="B60" s="2" t="s">
@@ -2595,10 +2613,10 @@
       <c r="D60" s="2">
         <v>29</v>
       </c>
-      <c r="E60" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F60" s="2" t="s">
+      <c r="E60" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F60" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G60" s="2">
@@ -2618,7 +2636,7 @@
       <c r="S60" s="4"/>
     </row>
     <row r="61" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="2">
+      <c r="A61" s="10">
         <v>341</v>
       </c>
       <c r="B61" s="2" t="s">
@@ -2630,10 +2648,10 @@
       <c r="D61" s="2">
         <v>57</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="E61" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="F61" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G61" s="2">
@@ -2653,22 +2671,22 @@
       <c r="S61" s="4"/>
     </row>
     <row r="62" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="9">
+      <c r="A62" s="12">
         <v>342</v>
       </c>
-      <c r="B62" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C62" s="9" t="s">
+      <c r="B62" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D62" s="2">
         <v>37</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F62" s="2" t="s">
+      <c r="E62" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F62" s="15" t="s">
         <v>10</v>
       </c>
       <c r="G62" s="2">
@@ -2688,22 +2706,22 @@
       <c r="S62" s="4"/>
     </row>
     <row r="63" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="9">
+      <c r="A63" s="12">
         <v>345</v>
       </c>
-      <c r="B63" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C63" s="9" t="s">
+      <c r="B63" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D63" s="2">
         <v>34</v>
       </c>
-      <c r="E63" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F63" s="2" t="s">
+      <c r="E63" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F63" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G63" s="2">
@@ -2723,7 +2741,7 @@
       <c r="S63" s="4"/>
     </row>
     <row r="64" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="6">
+      <c r="A64" s="11">
         <v>383</v>
       </c>
       <c r="B64" s="6" t="s">
@@ -2732,10 +2750,10 @@
       <c r="C64" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E64" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F64" s="2" t="s">
+      <c r="E64" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F64" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H64" s="5">
@@ -2752,7 +2770,7 @@
       <c r="S64" s="4"/>
     </row>
     <row r="65" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="6">
+      <c r="A65" s="11">
         <v>387</v>
       </c>
       <c r="B65" s="6" t="s">
@@ -2761,10 +2779,10 @@
       <c r="C65" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E65" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F65" s="2" t="s">
+      <c r="E65" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F65" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H65" s="5">
@@ -2781,7 +2799,7 @@
       <c r="S65" s="4"/>
     </row>
     <row r="66" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="6">
+      <c r="A66" s="11">
         <v>390</v>
       </c>
       <c r="B66" s="6" t="s">
@@ -2790,10 +2808,10 @@
       <c r="C66" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E66" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F66" s="2" t="s">
+      <c r="E66" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F66" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H66" s="5">
@@ -2810,7 +2828,7 @@
       <c r="S66" s="4"/>
     </row>
     <row r="67" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="6">
+      <c r="A67" s="11">
         <v>391</v>
       </c>
       <c r="B67" s="6" t="s">
@@ -2819,10 +2837,10 @@
       <c r="C67" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E67" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F67" s="2" t="s">
+      <c r="E67" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F67" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H67" s="5">
@@ -2839,7 +2857,7 @@
       <c r="S67" s="4"/>
     </row>
     <row r="68" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="6">
+      <c r="A68" s="11">
         <v>392</v>
       </c>
       <c r="B68" s="6" t="s">
@@ -2848,10 +2866,10 @@
       <c r="C68" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E68" s="2" t="s">
+      <c r="E68" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F68" s="2" t="s">
+      <c r="F68" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H68" s="5">
@@ -2868,7 +2886,7 @@
       <c r="S68" s="4"/>
     </row>
     <row r="69" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="6">
+      <c r="A69" s="11">
         <v>393</v>
       </c>
       <c r="B69" s="6" t="s">
@@ -2877,10 +2895,10 @@
       <c r="C69" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E69" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F69" s="2" t="s">
+      <c r="E69" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" s="15" t="s">
         <v>21</v>
       </c>
       <c r="H69" s="5">
@@ -2897,7 +2915,7 @@
       <c r="S69" s="4"/>
     </row>
     <row r="70" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="6">
+      <c r="A70" s="11">
         <v>394</v>
       </c>
       <c r="B70" s="6" t="s">
@@ -2906,10 +2924,10 @@
       <c r="C70" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E70" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F70" s="2" t="s">
+      <c r="E70" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F70" s="15" t="s">
         <v>21</v>
       </c>
       <c r="H70" s="5">
@@ -2926,7 +2944,7 @@
       <c r="S70" s="4"/>
     </row>
     <row r="71" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="6">
+      <c r="A71" s="11">
         <v>395</v>
       </c>
       <c r="B71" s="6" t="s">
@@ -2935,10 +2953,10 @@
       <c r="C71" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E71" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F71" s="2" t="s">
+      <c r="E71" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F71" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H71" s="5">
@@ -2955,7 +2973,7 @@
       <c r="S71" s="4"/>
     </row>
     <row r="72" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="6">
+      <c r="A72" s="11">
         <v>396</v>
       </c>
       <c r="B72" s="6" t="s">
@@ -2964,10 +2982,10 @@
       <c r="C72" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E72" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F72" s="2" t="s">
+      <c r="E72" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F72" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H72" s="5">
@@ -2984,7 +3002,7 @@
       <c r="S72" s="4"/>
     </row>
     <row r="73" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="6">
+      <c r="A73" s="11">
         <v>398</v>
       </c>
       <c r="B73" s="6" t="s">
@@ -2993,10 +3011,10 @@
       <c r="C73" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E73" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F73" s="2" t="s">
+      <c r="E73" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F73" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H73" s="5">
@@ -3013,7 +3031,7 @@
       <c r="S73" s="4"/>
     </row>
     <row r="74" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="6">
+      <c r="A74" s="11">
         <v>399</v>
       </c>
       <c r="B74" s="6" t="s">
@@ -3022,10 +3040,10 @@
       <c r="C74" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E74" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F74" s="2" t="s">
+      <c r="E74" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F74" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H74" s="5">
@@ -3042,15 +3060,15 @@
       <c r="S74" s="4"/>
     </row>
     <row r="75" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="10">
+      <c r="A75" s="12">
         <v>401</v>
       </c>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
-      <c r="E75" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F75" s="2" t="s">
+      <c r="B75" s="8"/>
+      <c r="C75" s="8"/>
+      <c r="E75" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F75" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H75" s="2">
@@ -3067,7 +3085,7 @@
       <c r="S75" s="4"/>
     </row>
     <row r="76" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="6">
+      <c r="A76" s="11">
         <v>402</v>
       </c>
       <c r="B76" s="6" t="s">
@@ -3076,10 +3094,10 @@
       <c r="C76" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E76" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F76" s="2" t="s">
+      <c r="E76" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F76" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H76" s="5">
@@ -3096,7 +3114,7 @@
       <c r="S76" s="4"/>
     </row>
     <row r="77" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="6">
+      <c r="A77" s="11">
         <v>403</v>
       </c>
       <c r="B77" s="6" t="s">
@@ -3105,10 +3123,10 @@
       <c r="C77" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E77" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F77" s="2" t="s">
+      <c r="E77" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F77" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H77" s="5">
@@ -3125,7 +3143,7 @@
       <c r="S77" s="4"/>
     </row>
     <row r="78" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="6">
+      <c r="A78" s="11">
         <v>404</v>
       </c>
       <c r="B78" s="6" t="s">
@@ -3134,10 +3152,10 @@
       <c r="C78" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E78" s="2" t="s">
+      <c r="E78" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F78" s="2" t="s">
+      <c r="F78" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H78" s="5">
@@ -3154,7 +3172,7 @@
       <c r="S78" s="4"/>
     </row>
     <row r="79" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="6">
+      <c r="A79" s="11">
         <v>405</v>
       </c>
       <c r="B79" s="6" t="s">
@@ -3163,10 +3181,10 @@
       <c r="C79" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E79" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F79" s="2" t="s">
+      <c r="E79" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F79" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H79" s="5">
@@ -3183,7 +3201,7 @@
       <c r="S79" s="4"/>
     </row>
     <row r="80" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="6">
+      <c r="A80" s="11">
         <v>406</v>
       </c>
       <c r="B80" s="6" t="s">
@@ -3192,10 +3210,10 @@
       <c r="C80" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E80" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F80" s="2" t="s">
+      <c r="E80" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F80" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H80" s="5">
@@ -3212,7 +3230,7 @@
       <c r="S80" s="4"/>
     </row>
     <row r="81" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="6">
+      <c r="A81" s="11">
         <v>407</v>
       </c>
       <c r="B81" s="6" t="s">
@@ -3221,10 +3239,10 @@
       <c r="C81" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E81" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F81" s="2" t="s">
+      <c r="E81" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F81" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H81" s="5">
@@ -3241,19 +3259,19 @@
       <c r="S81" s="4"/>
     </row>
     <row r="82" spans="1:19" ht="20" x14ac:dyDescent="0.25">
-      <c r="A82" s="8">
+      <c r="A82" s="13">
         <v>408</v>
       </c>
-      <c r="B82" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C82" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F82" s="2" t="s">
+      <c r="B82" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F82" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H82" s="5">
@@ -3270,19 +3288,19 @@
       <c r="S82" s="4"/>
     </row>
     <row r="83" spans="1:19" ht="20" x14ac:dyDescent="0.25">
-      <c r="A83" s="8">
+      <c r="A83" s="13">
         <v>409</v>
       </c>
-      <c r="B83" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C83" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F83" s="2" t="s">
+      <c r="B83" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F83" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H83" s="5">
@@ -3299,19 +3317,19 @@
       <c r="S83" s="4"/>
     </row>
     <row r="84" spans="1:19" ht="20" x14ac:dyDescent="0.25">
-      <c r="A84" s="8">
+      <c r="A84" s="13">
         <v>410</v>
       </c>
-      <c r="B84" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C84" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E84" s="2" t="s">
+      <c r="B84" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F84" s="2" t="s">
+      <c r="F84" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H84" s="5">
@@ -3328,13 +3346,13 @@
       <c r="S84" s="4"/>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A85" s="7">
+      <c r="A85" s="10">
         <v>411</v>
       </c>
-      <c r="E85" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F85" s="2" t="s">
+      <c r="E85" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F85" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H85" s="2">
@@ -3351,13 +3369,13 @@
       <c r="S85" s="4"/>
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A86" s="7">
+      <c r="A86" s="10">
         <v>413</v>
       </c>
-      <c r="E86" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F86" s="2" t="s">
+      <c r="E86" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F86" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H86" s="2">
@@ -3374,13 +3392,13 @@
       <c r="S86" s="4"/>
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A87" s="7">
+      <c r="A87" s="10">
         <v>415</v>
       </c>
-      <c r="E87" s="2" t="s">
+      <c r="E87" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F87" s="2" t="s">
+      <c r="F87" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H87" s="2">
@@ -3397,13 +3415,13 @@
       <c r="S87" s="4"/>
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A88" s="7">
+      <c r="A88" s="10">
         <v>416</v>
       </c>
-      <c r="E88" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F88" s="2" t="s">
+      <c r="E88" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F88" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H88" s="2">
@@ -3420,13 +3438,13 @@
       <c r="S88" s="4"/>
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A89" s="7">
+      <c r="A89" s="10">
         <v>417</v>
       </c>
-      <c r="E89" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F89" s="2" t="s">
+      <c r="E89" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F89" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H89" s="2">
@@ -3443,13 +3461,13 @@
       <c r="S89" s="4"/>
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A90" s="7">
+      <c r="A90" s="10">
         <v>418</v>
       </c>
-      <c r="E90" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F90" s="2" t="s">
+      <c r="E90" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F90" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H90" s="2">
@@ -3466,13 +3484,13 @@
       <c r="S90" s="4"/>
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A91" s="7">
+      <c r="A91" s="10">
         <v>418</v>
       </c>
-      <c r="E91" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F91" s="2" t="s">
+      <c r="E91" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F91" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H91" s="2">
@@ -3489,13 +3507,13 @@
       <c r="S91" s="4"/>
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A92" s="7">
+      <c r="A92" s="10">
         <v>419</v>
       </c>
-      <c r="E92" s="2" t="s">
+      <c r="E92" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F92" s="2" t="s">
+      <c r="F92" s="15" t="s">
         <v>16</v>
       </c>
       <c r="H92" s="2">
@@ -3512,13 +3530,13 @@
       <c r="S92" s="4"/>
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A93" s="7">
+      <c r="A93" s="10">
         <v>420</v>
       </c>
-      <c r="E93" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F93" s="2" t="s">
+      <c r="E93" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F93" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H93" s="2">
@@ -3535,13 +3553,13 @@
       <c r="S93" s="4"/>
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A94" s="7">
+      <c r="A94" s="10">
         <v>421</v>
       </c>
-      <c r="E94" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F94" s="2" t="s">
+      <c r="E94" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F94" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H94" s="2">
@@ -3558,13 +3576,13 @@
       <c r="S94" s="4"/>
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A95" s="7">
+      <c r="A95" s="10">
         <v>424</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E95" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F95" s="2" t="s">
+      <c r="F95" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H95" s="2">
@@ -3581,13 +3599,13 @@
       <c r="S95" s="4"/>
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A96" s="7">
+      <c r="A96" s="10">
         <v>425</v>
       </c>
-      <c r="E96" s="2" t="s">
+      <c r="E96" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F96" s="2" t="s">
+      <c r="F96" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H96" s="2">
@@ -3604,13 +3622,13 @@
       <c r="S96" s="4"/>
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A97" s="7">
+      <c r="A97" s="10">
         <v>426</v>
       </c>
-      <c r="E97" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F97" s="2" t="s">
+      <c r="E97" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F97" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H97" s="2">
@@ -3627,13 +3645,13 @@
       <c r="S97" s="4"/>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A98" s="7">
+      <c r="A98" s="10">
         <v>427</v>
       </c>
-      <c r="E98" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F98" s="2" t="s">
+      <c r="E98" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F98" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H98" s="2">
@@ -3650,13 +3668,13 @@
       <c r="S98" s="4"/>
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A99" s="7">
+      <c r="A99" s="10">
         <v>428</v>
       </c>
-      <c r="E99" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F99" s="2" t="s">
+      <c r="E99" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F99" s="15" t="s">
         <v>16</v>
       </c>
       <c r="H99" s="2">
@@ -3673,13 +3691,13 @@
       <c r="S99" s="4"/>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A100" s="7">
+      <c r="A100" s="10">
         <v>429</v>
       </c>
-      <c r="E100" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F100" s="2" t="s">
+      <c r="E100" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F100" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H100" s="2">
@@ -3696,13 +3714,13 @@
       <c r="S100" s="4"/>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A101" s="7">
+      <c r="A101" s="10">
         <v>430</v>
       </c>
-      <c r="E101" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F101" s="2" t="s">
+      <c r="E101" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F101" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H101" s="2">
@@ -3719,13 +3737,13 @@
       <c r="S101" s="4"/>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A102" s="7">
+      <c r="A102" s="10">
         <v>431</v>
       </c>
-      <c r="E102" s="2" t="s">
+      <c r="E102" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F102" s="2" t="s">
+      <c r="F102" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H102" s="2">
@@ -3742,13 +3760,13 @@
       <c r="S102" s="4"/>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A103" s="7">
+      <c r="A103" s="10">
         <v>432</v>
       </c>
-      <c r="E103" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F103" s="2" t="s">
+      <c r="E103" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F103" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H103" s="2">
@@ -3765,13 +3783,13 @@
       <c r="S103" s="4"/>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A104" s="7">
+      <c r="A104" s="10">
         <v>433</v>
       </c>
-      <c r="E104" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F104" s="2" t="s">
+      <c r="E104" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F104" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H104" s="2">
@@ -3788,13 +3806,13 @@
       <c r="S104" s="4"/>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A105" s="7">
+      <c r="A105" s="10">
         <v>434</v>
       </c>
-      <c r="E105" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F105" s="2" t="s">
+      <c r="E105" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F105" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H105" s="2">
@@ -3811,13 +3829,13 @@
       <c r="S105" s="4"/>
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A106" s="7">
+      <c r="A106" s="10">
         <v>435</v>
       </c>
-      <c r="E106" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F106" s="2" t="s">
+      <c r="E106" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F106" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H106" s="2">
@@ -3834,13 +3852,13 @@
       <c r="S106" s="4"/>
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A107" s="7">
+      <c r="A107" s="10">
         <v>436</v>
       </c>
-      <c r="E107" s="2" t="s">
+      <c r="E107" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F107" s="2" t="s">
+      <c r="F107" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H107" s="2">
@@ -3857,13 +3875,13 @@
       <c r="S107" s="4"/>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A108" s="7">
+      <c r="A108" s="10">
         <v>437</v>
       </c>
-      <c r="E108" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F108" s="2" t="s">
+      <c r="E108" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F108" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H108" s="2">
@@ -3880,13 +3898,13 @@
       <c r="S108" s="4"/>
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A109" s="7">
+      <c r="A109" s="10">
         <v>438</v>
       </c>
-      <c r="E109" s="2" t="s">
+      <c r="E109" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F109" s="2" t="s">
+      <c r="F109" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H109" s="2">
@@ -3903,13 +3921,13 @@
       <c r="S109" s="4"/>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A110" s="7">
+      <c r="A110" s="10">
         <v>439</v>
       </c>
-      <c r="E110" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F110" s="2" t="s">
+      <c r="E110" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F110" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H110" s="2">
@@ -3926,13 +3944,13 @@
       <c r="S110" s="4"/>
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A111" s="7">
+      <c r="A111" s="10">
         <v>439</v>
       </c>
-      <c r="E111" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F111" s="2" t="s">
+      <c r="E111" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F111" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H111" s="2">
@@ -3949,13 +3967,13 @@
       <c r="S111" s="4"/>
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A112" s="7">
+      <c r="A112" s="10">
         <v>440</v>
       </c>
-      <c r="E112" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F112" s="2" t="s">
+      <c r="E112" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F112" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H112" s="2">
@@ -3972,13 +3990,13 @@
       <c r="S112" s="4"/>
     </row>
     <row r="113" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A113" s="7">
+      <c r="A113" s="10">
         <v>441</v>
       </c>
-      <c r="E113" s="2" t="s">
+      <c r="E113" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F113" s="2" t="s">
+      <c r="F113" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H113" s="2">
@@ -3995,13 +4013,13 @@
       <c r="S113" s="4"/>
     </row>
     <row r="114" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A114" s="7">
+      <c r="A114" s="10">
         <v>442</v>
       </c>
-      <c r="E114" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F114" s="2" t="s">
+      <c r="E114" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F114" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H114" s="2">
@@ -4018,13 +4036,13 @@
       <c r="S114" s="4"/>
     </row>
     <row r="115" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A115" s="7">
+      <c r="A115" s="10">
         <v>443</v>
       </c>
-      <c r="E115" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F115" s="2" t="s">
+      <c r="E115" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F115" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H115" s="2">
@@ -4041,13 +4059,13 @@
       <c r="S115" s="4"/>
     </row>
     <row r="116" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A116" s="7">
+      <c r="A116" s="10">
         <v>444</v>
       </c>
-      <c r="E116" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F116" s="2" t="s">
+      <c r="E116" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F116" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H116" s="2">
@@ -4064,13 +4082,13 @@
       <c r="S116" s="4"/>
     </row>
     <row r="117" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A117" s="7">
+      <c r="A117" s="10">
         <v>445</v>
       </c>
-      <c r="E117" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F117" s="2" t="s">
+      <c r="E117" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F117" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H117" s="2">
@@ -4087,13 +4105,13 @@
       <c r="S117" s="4"/>
     </row>
     <row r="118" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A118" s="7">
+      <c r="A118" s="10">
         <v>446</v>
       </c>
-      <c r="E118" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F118" s="2" t="s">
+      <c r="E118" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F118" s="15" t="s">
         <v>13</v>
       </c>
       <c r="H118" s="2">
@@ -4110,13 +4128,13 @@
       <c r="S118" s="4"/>
     </row>
     <row r="119" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A119" s="7">
+      <c r="A119" s="10">
         <v>448</v>
       </c>
-      <c r="E119" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F119" s="2" t="s">
+      <c r="E119" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F119" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H119" s="2">
@@ -4133,13 +4151,13 @@
       <c r="S119" s="4"/>
     </row>
     <row r="120" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A120" s="7">
+      <c r="A120" s="10">
         <v>449</v>
       </c>
-      <c r="E120" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F120" s="2" t="s">
+      <c r="E120" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F120" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H120" s="2">
@@ -4156,13 +4174,13 @@
       <c r="S120" s="4"/>
     </row>
     <row r="121" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A121" s="7">
+      <c r="A121" s="10">
         <v>450</v>
       </c>
-      <c r="E121" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F121" s="2" t="s">
+      <c r="E121" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F121" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H121" s="2">
@@ -4179,13 +4197,13 @@
       <c r="S121" s="4"/>
     </row>
     <row r="122" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A122" s="7">
+      <c r="A122" s="10">
         <v>451</v>
       </c>
-      <c r="E122" s="2" t="s">
+      <c r="E122" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F122" s="2" t="s">
+      <c r="F122" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H122" s="2">
@@ -4202,13 +4220,13 @@
       <c r="S122" s="4"/>
     </row>
     <row r="123" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A123" s="7">
+      <c r="A123" s="10">
         <v>452</v>
       </c>
-      <c r="E123" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F123" s="2" t="s">
+      <c r="E123" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F123" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H123" s="2">
@@ -4225,13 +4243,13 @@
       <c r="S123" s="4"/>
     </row>
     <row r="124" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A124" s="7">
+      <c r="A124" s="10">
         <v>454</v>
       </c>
-      <c r="E124" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F124" s="2" t="s">
+      <c r="E124" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F124" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H124" s="2">
@@ -4248,13 +4266,13 @@
       <c r="S124" s="4"/>
     </row>
     <row r="125" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A125" s="7">
+      <c r="A125" s="10">
         <v>455</v>
       </c>
-      <c r="E125" s="2" t="s">
+      <c r="E125" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F125" s="2" t="s">
+      <c r="F125" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H125" s="2">
@@ -4271,13 +4289,13 @@
       <c r="S125" s="4"/>
     </row>
     <row r="126" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A126" s="7">
+      <c r="A126" s="10">
         <v>456</v>
       </c>
-      <c r="E126" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F126" s="2" t="s">
+      <c r="E126" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F126" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H126" s="2">
@@ -4294,13 +4312,13 @@
       <c r="S126" s="4"/>
     </row>
     <row r="127" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A127" s="7">
+      <c r="A127" s="10">
         <v>458</v>
       </c>
-      <c r="E127" s="2" t="s">
+      <c r="E127" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F127" s="2" t="s">
+      <c r="F127" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H127" s="2">
@@ -4317,13 +4335,13 @@
       <c r="S127" s="4"/>
     </row>
     <row r="128" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A128" s="7">
+      <c r="A128" s="10">
         <v>459</v>
       </c>
-      <c r="E128" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F128" s="2" t="s">
+      <c r="E128" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F128" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H128" s="2">
@@ -4340,13 +4358,13 @@
       <c r="S128" s="4"/>
     </row>
     <row r="129" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A129" s="7">
+      <c r="A129" s="10">
         <v>462</v>
       </c>
-      <c r="E129" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F129" s="2" t="s">
+      <c r="E129" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F129" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H129" s="2">
@@ -4363,13 +4381,13 @@
       <c r="S129" s="4"/>
     </row>
     <row r="130" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A130" s="7">
+      <c r="A130" s="10">
         <v>465</v>
       </c>
-      <c r="E130" s="2" t="s">
+      <c r="E130" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F130" s="2" t="s">
+      <c r="F130" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H130" s="2">
@@ -4386,13 +4404,13 @@
       <c r="S130" s="4"/>
     </row>
     <row r="131" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A131" s="7">
+      <c r="A131" s="10">
         <v>468</v>
       </c>
-      <c r="E131" s="2" t="s">
+      <c r="E131" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F131" s="2" t="s">
+      <c r="F131" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H131" s="2">
@@ -4409,13 +4427,13 @@
       <c r="S131" s="4"/>
     </row>
     <row r="132" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A132" s="7">
+      <c r="A132" s="10">
         <v>471</v>
       </c>
-      <c r="E132" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F132" s="2" t="s">
+      <c r="E132" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F132" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H132" s="2">
@@ -4432,13 +4450,13 @@
       <c r="S132" s="4"/>
     </row>
     <row r="133" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A133" s="7">
+      <c r="A133" s="10">
         <v>472</v>
       </c>
-      <c r="E133" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F133" s="2" t="s">
+      <c r="E133" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F133" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H133" s="2">
@@ -4455,13 +4473,13 @@
       <c r="S133" s="4"/>
     </row>
     <row r="134" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A134" s="7">
+      <c r="A134" s="10">
         <v>473</v>
       </c>
-      <c r="E134" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F134" s="2" t="s">
+      <c r="E134" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F134" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H134" s="2">
@@ -4478,13 +4496,13 @@
       <c r="S134" s="4"/>
     </row>
     <row r="135" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A135" s="7">
+      <c r="A135" s="10">
         <v>474</v>
       </c>
-      <c r="E135" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F135" s="2" t="s">
+      <c r="E135" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F135" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H135" s="2">
@@ -4501,13 +4519,13 @@
       <c r="S135" s="4"/>
     </row>
     <row r="136" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A136" s="7">
+      <c r="A136" s="10">
         <v>477</v>
       </c>
-      <c r="E136" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F136" s="2" t="s">
+      <c r="E136" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F136" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H136" s="2">
@@ -4524,13 +4542,13 @@
       <c r="S136" s="4"/>
     </row>
     <row r="137" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A137" s="7">
+      <c r="A137" s="10">
         <v>478</v>
       </c>
-      <c r="E137" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F137" s="2" t="s">
+      <c r="E137" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F137" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H137" s="2">
@@ -4547,13 +4565,13 @@
       <c r="S137" s="4"/>
     </row>
     <row r="138" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A138" s="7">
+      <c r="A138" s="10">
         <v>479</v>
       </c>
-      <c r="E138" s="2" t="s">
+      <c r="E138" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F138" s="2" t="s">
+      <c r="F138" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H138" s="2">
@@ -4570,13 +4588,13 @@
       <c r="S138" s="4"/>
     </row>
     <row r="139" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A139" s="7">
+      <c r="A139" s="10">
         <v>482</v>
       </c>
-      <c r="E139" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F139" s="2" t="s">
+      <c r="E139" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F139" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H139" s="2">
@@ -4593,13 +4611,13 @@
       <c r="S139" s="4"/>
     </row>
     <row r="140" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A140" s="7">
+      <c r="A140" s="10">
         <v>483</v>
       </c>
-      <c r="E140" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F140" s="2" t="s">
+      <c r="E140" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F140" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H140" s="2">
@@ -4616,13 +4634,13 @@
       <c r="S140" s="4"/>
     </row>
     <row r="141" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A141" s="7">
+      <c r="A141" s="10">
         <v>484</v>
       </c>
-      <c r="E141" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F141" s="2" t="s">
+      <c r="E141" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F141" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H141" s="2">
@@ -4639,13 +4657,13 @@
       <c r="S141" s="4"/>
     </row>
     <row r="142" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A142" s="7">
+      <c r="A142" s="10">
         <v>485</v>
       </c>
-      <c r="E142" s="2" t="s">
+      <c r="E142" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F142" s="2" t="s">
+      <c r="F142" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H142" s="2">
@@ -4660,13 +4678,13 @@
       </c>
     </row>
     <row r="143" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A143" s="7">
+      <c r="A143" s="10">
         <v>487</v>
       </c>
-      <c r="E143" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F143" s="2" t="s">
+      <c r="E143" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F143" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H143" s="2">
@@ -4681,13 +4699,13 @@
       </c>
     </row>
     <row r="144" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A144" s="7">
+      <c r="A144" s="10">
         <v>488</v>
       </c>
-      <c r="E144" s="2" t="s">
+      <c r="E144" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F144" s="2" t="s">
+      <c r="F144" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H144" s="2">
@@ -4702,13 +4720,13 @@
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A145" s="7">
+      <c r="A145" s="10">
         <v>489</v>
       </c>
-      <c r="E145" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F145" s="2" t="s">
+      <c r="E145" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F145" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H145" s="2">
@@ -4723,13 +4741,13 @@
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A146" s="7">
+      <c r="A146" s="10">
         <v>490</v>
       </c>
-      <c r="E146" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F146" s="2" t="s">
+      <c r="E146" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F146" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H146" s="2">
@@ -4744,13 +4762,13 @@
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A147" s="7">
+      <c r="A147" s="10">
         <v>491</v>
       </c>
-      <c r="E147" s="2" t="s">
+      <c r="E147" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F147" s="2" t="s">
+      <c r="F147" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H147" s="2">
@@ -4765,13 +4783,13 @@
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A148" s="7">
+      <c r="A148" s="10">
         <v>493</v>
       </c>
-      <c r="E148" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F148" s="2" t="s">
+      <c r="E148" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F148" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H148" s="2">
@@ -4786,13 +4804,13 @@
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A149" s="7">
+      <c r="A149" s="10">
         <v>494</v>
       </c>
-      <c r="E149" s="2" t="s">
+      <c r="E149" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F149" s="2" t="s">
+      <c r="F149" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H149" s="2">
@@ -4807,13 +4825,13 @@
       </c>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A150" s="7">
+      <c r="A150" s="10">
         <v>498</v>
       </c>
-      <c r="E150" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F150" s="2" t="s">
+      <c r="E150" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F150" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H150" s="2">
@@ -4828,13 +4846,13 @@
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A151" s="7">
+      <c r="A151" s="10">
         <v>499</v>
       </c>
-      <c r="E151" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F151" s="2" t="s">
+      <c r="E151" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F151" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H151" s="2">
@@ -4849,13 +4867,13 @@
       </c>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A152" s="7">
+      <c r="A152" s="10">
         <v>500</v>
       </c>
-      <c r="E152" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F152" s="2" t="s">
+      <c r="E152" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F152" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H152" s="2">
@@ -4870,13 +4888,13 @@
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A153" s="7">
+      <c r="A153" s="10">
         <v>501</v>
       </c>
-      <c r="E153" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F153" s="2" t="s">
+      <c r="E153" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F153" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H153" s="2">
@@ -4891,13 +4909,13 @@
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A154" s="7">
+      <c r="A154" s="10">
         <v>502</v>
       </c>
-      <c r="E154" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F154" s="2" t="s">
+      <c r="E154" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F154" s="15" t="s">
         <v>18</v>
       </c>
       <c r="H154" s="2">
@@ -4912,13 +4930,13 @@
       </c>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A155" s="7">
+      <c r="A155" s="10">
         <v>505</v>
       </c>
-      <c r="E155" s="2" t="s">
+      <c r="E155" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F155" s="2" t="s">
+      <c r="F155" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H155" s="2">
@@ -4933,13 +4951,13 @@
       </c>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A156" s="7">
+      <c r="A156" s="10">
         <v>506</v>
       </c>
-      <c r="E156" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F156" s="2" t="s">
+      <c r="E156" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F156" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H156" s="2">
@@ -4954,13 +4972,13 @@
       </c>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A157" s="7">
+      <c r="A157" s="10">
         <v>508</v>
       </c>
-      <c r="E157" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F157" s="2" t="s">
+      <c r="E157" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F157" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H157" s="2">
@@ -4975,13 +4993,13 @@
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A158" s="7">
+      <c r="A158" s="10">
         <v>509</v>
       </c>
-      <c r="E158" s="2" t="s">
+      <c r="E158" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F158" s="2" t="s">
+      <c r="F158" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H158" s="2">
@@ -4996,13 +5014,13 @@
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A159" s="7">
+      <c r="A159" s="10">
         <v>510</v>
       </c>
-      <c r="E159" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F159" s="2" t="s">
+      <c r="E159" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F159" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H159" s="2">
@@ -5017,13 +5035,13 @@
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A160" s="7">
+      <c r="A160" s="10">
         <v>511</v>
       </c>
-      <c r="E160" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F160" s="2" t="s">
+      <c r="E160" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F160" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H160" s="2">
@@ -5038,13 +5056,13 @@
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A161" s="7">
+      <c r="A161" s="10">
         <v>512</v>
       </c>
-      <c r="E161" s="2" t="s">
+      <c r="E161" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F161" s="2" t="s">
+      <c r="F161" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H161" s="2">
@@ -5059,13 +5077,13 @@
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A162" s="7">
+      <c r="A162" s="10">
         <v>514</v>
       </c>
-      <c r="E162" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F162" s="2" t="s">
+      <c r="E162" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F162" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H162" s="2">
@@ -5080,13 +5098,13 @@
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A163" s="7">
+      <c r="A163" s="10">
         <v>515</v>
       </c>
-      <c r="E163" s="2" t="s">
+      <c r="E163" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F163" s="2" t="s">
+      <c r="F163" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H163" s="2">
@@ -5101,13 +5119,13 @@
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A164" s="7">
+      <c r="A164" s="10">
         <v>516</v>
       </c>
-      <c r="E164" s="2" t="s">
+      <c r="E164" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F164" s="2" t="s">
+      <c r="F164" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H164" s="2">
@@ -5122,13 +5140,13 @@
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A165" s="7">
+      <c r="A165" s="10">
         <v>517</v>
       </c>
-      <c r="E165" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F165" s="2" t="s">
+      <c r="E165" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F165" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H165" s="2">
@@ -5143,13 +5161,13 @@
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A166" s="7">
+      <c r="A166" s="10">
         <v>518</v>
       </c>
-      <c r="E166" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F166" s="2" t="s">
+      <c r="E166" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F166" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H166" s="2">
@@ -5164,13 +5182,13 @@
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A167" s="7">
+      <c r="A167" s="10">
         <v>519</v>
       </c>
-      <c r="E167" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F167" s="2" t="s">
+      <c r="E167" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F167" s="15" t="s">
         <v>13</v>
       </c>
       <c r="H167" s="2">
@@ -5185,13 +5203,13 @@
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A168" s="7">
+      <c r="A168" s="10">
         <v>520</v>
       </c>
-      <c r="E168" s="2" t="s">
+      <c r="E168" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F168" s="2" t="s">
+      <c r="F168" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H168" s="2">
@@ -5206,13 +5224,13 @@
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A169" s="7">
+      <c r="A169" s="10">
         <v>521</v>
       </c>
-      <c r="E169" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F169" s="2" t="s">
+      <c r="E169" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F169" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H169" s="2">
@@ -5227,13 +5245,13 @@
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A170" s="7">
+      <c r="A170" s="10">
         <v>522</v>
       </c>
-      <c r="E170" s="2" t="s">
+      <c r="E170" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F170" s="2" t="s">
+      <c r="F170" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H170" s="2">
@@ -5248,13 +5266,13 @@
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A171" s="7">
+      <c r="A171" s="10">
         <v>523</v>
       </c>
-      <c r="E171" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F171" s="2" t="s">
+      <c r="E171" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F171" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H171" s="2">
@@ -5269,13 +5287,13 @@
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A172" s="7">
+      <c r="A172" s="10">
         <v>524</v>
       </c>
-      <c r="E172" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F172" s="2" t="s">
+      <c r="E172" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F172" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H172" s="2">
@@ -5290,13 +5308,13 @@
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A173" s="7">
+      <c r="A173" s="10">
         <v>526</v>
       </c>
-      <c r="E173" s="2" t="s">
+      <c r="E173" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F173" s="2" t="s">
+      <c r="F173" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H173" s="2">
@@ -5311,13 +5329,13 @@
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A174" s="7">
+      <c r="A174" s="10">
         <v>528</v>
       </c>
-      <c r="E174" s="2" t="s">
+      <c r="E174" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F174" s="2" t="s">
+      <c r="F174" s="15" t="s">
         <v>13</v>
       </c>
       <c r="H174" s="2">
@@ -5332,13 +5350,13 @@
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A175" s="7">
+      <c r="A175" s="10">
         <v>529</v>
       </c>
-      <c r="E175" s="2" t="s">
+      <c r="E175" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F175" s="2" t="s">
+      <c r="F175" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H175" s="2">
@@ -5353,13 +5371,13 @@
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A176" s="7">
+      <c r="A176" s="10">
         <v>530</v>
       </c>
-      <c r="E176" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F176" s="2" t="s">
+      <c r="E176" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F176" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H176" s="2">
@@ -5374,13 +5392,13 @@
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A177" s="7">
+      <c r="A177" s="10">
         <v>531</v>
       </c>
-      <c r="E177" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F177" s="2" t="s">
+      <c r="E177" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F177" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H177" s="2">
@@ -5395,13 +5413,13 @@
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A178" s="7">
+      <c r="A178" s="10">
         <v>533</v>
       </c>
-      <c r="E178" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F178" s="2" t="s">
+      <c r="E178" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F178" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H178" s="2">
@@ -5416,13 +5434,13 @@
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A179" s="7">
+      <c r="A179" s="10">
         <v>534</v>
       </c>
-      <c r="E179" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F179" s="2" t="s">
+      <c r="E179" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F179" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H179" s="2">
@@ -5437,13 +5455,13 @@
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A180" s="7">
+      <c r="A180" s="10">
         <v>536</v>
       </c>
-      <c r="E180" s="2" t="s">
+      <c r="E180" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F180" s="2" t="s">
+      <c r="F180" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H180" s="2">
@@ -5458,13 +5476,13 @@
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A181" s="7">
+      <c r="A181" s="10">
         <v>537</v>
       </c>
-      <c r="E181" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F181" s="2" t="s">
+      <c r="E181" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F181" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H181" s="2">
@@ -5479,13 +5497,13 @@
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A182" s="7">
+      <c r="A182" s="10">
         <v>538</v>
       </c>
-      <c r="E182" s="2" t="s">
+      <c r="E182" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F182" s="2" t="s">
+      <c r="F182" s="15" t="s">
         <v>18</v>
       </c>
       <c r="H182" s="2">
@@ -5500,13 +5518,13 @@
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A183" s="7">
+      <c r="A183" s="10">
         <v>539</v>
       </c>
-      <c r="E183" s="2" t="s">
+      <c r="E183" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F183" s="2" t="s">
+      <c r="F183" s="15" t="s">
         <v>13</v>
       </c>
       <c r="H183" s="2">
@@ -5521,13 +5539,13 @@
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A184" s="7">
+      <c r="A184" s="10">
         <v>540</v>
       </c>
-      <c r="E184" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F184" s="2" t="s">
+      <c r="E184" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F184" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H184" s="2">
@@ -5542,13 +5560,13 @@
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A185" s="7">
+      <c r="A185" s="10">
         <v>544</v>
       </c>
-      <c r="E185" s="2" t="s">
+      <c r="E185" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F185" s="2" t="s">
+      <c r="F185" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H185" s="2">
@@ -5563,13 +5581,13 @@
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A186" s="7">
+      <c r="A186" s="10">
         <v>545</v>
       </c>
-      <c r="E186" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F186" s="2" t="s">
+      <c r="E186" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F186" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H186" s="2">
@@ -5584,13 +5602,13 @@
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A187" s="7">
+      <c r="A187" s="10">
         <v>546</v>
       </c>
-      <c r="E187" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F187" s="2" t="s">
+      <c r="E187" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F187" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H187" s="2">
@@ -5605,13 +5623,13 @@
       </c>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A188" s="7">
+      <c r="A188" s="10">
         <v>548</v>
       </c>
-      <c r="E188" s="2" t="s">
+      <c r="E188" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F188" s="2" t="s">
+      <c r="F188" s="15" t="s">
         <v>18</v>
       </c>
       <c r="H188" s="2">
@@ -5626,13 +5644,13 @@
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A189" s="7">
+      <c r="A189" s="10">
         <v>549</v>
       </c>
-      <c r="E189" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F189" s="2" t="s">
+      <c r="E189" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F189" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H189" s="2">
@@ -5647,13 +5665,13 @@
       </c>
     </row>
     <row r="190" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A190" s="7">
+      <c r="A190" s="10">
         <v>550</v>
       </c>
-      <c r="E190" s="2" t="s">
+      <c r="E190" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F190" s="2" t="s">
+      <c r="F190" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H190" s="2">
@@ -5668,13 +5686,13 @@
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A191" s="7">
+      <c r="A191" s="10">
         <v>551</v>
       </c>
-      <c r="E191" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F191" s="2" t="s">
+      <c r="E191" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F191" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H191" s="2">
@@ -5689,13 +5707,13 @@
       </c>
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A192" s="7">
+      <c r="A192" s="10">
         <v>552</v>
       </c>
-      <c r="E192" s="2" t="s">
+      <c r="E192" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F192" s="2" t="s">
+      <c r="F192" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H192" s="2">
@@ -5710,13 +5728,13 @@
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A193" s="7">
+      <c r="A193" s="10">
         <v>553</v>
       </c>
-      <c r="E193" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F193" s="2" t="s">
+      <c r="E193" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F193" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H193" s="2">
@@ -5731,13 +5749,13 @@
       </c>
     </row>
     <row r="194" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A194" s="7">
+      <c r="A194" s="10">
         <v>554</v>
       </c>
-      <c r="E194" s="2" t="s">
+      <c r="E194" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F194" s="2" t="s">
+      <c r="F194" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H194" s="2">
@@ -5752,13 +5770,13 @@
       </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A195" s="7">
+      <c r="A195" s="10">
         <v>555</v>
       </c>
-      <c r="E195" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F195" s="2" t="s">
+      <c r="E195" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F195" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H195" s="2">
@@ -5773,13 +5791,13 @@
       </c>
     </row>
     <row r="196" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A196" s="7">
+      <c r="A196" s="10">
         <v>560</v>
       </c>
-      <c r="E196" s="2" t="s">
+      <c r="E196" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F196" s="2" t="s">
+      <c r="F196" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H196" s="2">
@@ -5794,13 +5812,13 @@
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A197" s="7">
+      <c r="A197" s="10">
         <v>563</v>
       </c>
-      <c r="E197" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F197" s="2" t="s">
+      <c r="E197" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F197" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H197" s="2">
@@ -5815,13 +5833,13 @@
       </c>
     </row>
     <row r="198" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A198" s="7">
+      <c r="A198" s="10">
         <v>564</v>
       </c>
-      <c r="E198" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F198" s="2" t="s">
+      <c r="E198" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F198" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H198" s="2">
@@ -5836,13 +5854,13 @@
       </c>
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A199" s="7">
+      <c r="A199" s="10">
         <v>565</v>
       </c>
-      <c r="E199" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F199" s="2" t="s">
+      <c r="E199" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F199" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H199" s="2">
@@ -5857,13 +5875,13 @@
       </c>
     </row>
     <row r="200" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A200" s="7">
+      <c r="A200" s="10">
         <v>566</v>
       </c>
-      <c r="E200" s="2" t="s">
+      <c r="E200" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F200" s="2" t="s">
+      <c r="F200" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H200" s="2">
@@ -5878,13 +5896,13 @@
       </c>
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A201" s="7">
+      <c r="A201" s="10">
         <v>567</v>
       </c>
-      <c r="E201" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F201" s="2" t="s">
+      <c r="E201" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F201" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H201" s="2">
@@ -5899,13 +5917,13 @@
       </c>
     </row>
     <row r="202" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A202" s="7">
+      <c r="A202" s="10">
         <v>568</v>
       </c>
-      <c r="E202" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F202" s="2" t="s">
+      <c r="E202" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F202" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H202" s="2">
@@ -5920,13 +5938,13 @@
       </c>
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A203" s="7">
+      <c r="A203" s="10">
         <v>569</v>
       </c>
-      <c r="E203" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F203" s="2" t="s">
+      <c r="E203" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F203" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H203" s="2">
@@ -5941,13 +5959,13 @@
       </c>
     </row>
     <row r="204" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A204" s="7">
+      <c r="A204" s="10">
         <v>570</v>
       </c>
-      <c r="E204" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F204" s="2" t="s">
+      <c r="E204" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F204" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H204" s="2">
@@ -5962,13 +5980,13 @@
       </c>
     </row>
     <row r="205" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A205" s="7">
+      <c r="A205" s="10">
         <v>572</v>
       </c>
-      <c r="E205" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F205" s="2" t="s">
+      <c r="E205" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F205" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H205" s="2">
@@ -5983,13 +6001,13 @@
       </c>
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A206" s="7">
+      <c r="A206" s="10">
         <v>573</v>
       </c>
-      <c r="E206" s="2" t="s">
+      <c r="E206" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F206" s="2" t="s">
+      <c r="F206" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H206" s="2">
@@ -6004,13 +6022,13 @@
       </c>
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A207" s="7">
+      <c r="A207" s="10">
         <v>575</v>
       </c>
-      <c r="E207" s="2" t="s">
+      <c r="E207" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F207" s="2" t="s">
+      <c r="F207" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H207" s="2">
@@ -6025,13 +6043,13 @@
       </c>
     </row>
     <row r="208" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A208" s="7">
+      <c r="A208" s="10">
         <v>576</v>
       </c>
-      <c r="E208" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F208" s="2" t="s">
+      <c r="E208" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F208" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H208" s="2">
@@ -6046,13 +6064,13 @@
       </c>
     </row>
     <row r="209" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A209" s="7">
+      <c r="A209" s="10">
         <v>577</v>
       </c>
-      <c r="E209" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F209" s="2" t="s">
+      <c r="E209" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F209" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H209" s="2">
@@ -6067,13 +6085,13 @@
       </c>
     </row>
     <row r="210" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A210" s="7">
+      <c r="A210" s="10">
         <v>578</v>
       </c>
-      <c r="E210" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F210" s="2" t="s">
+      <c r="E210" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F210" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H210" s="2">
@@ -6088,13 +6106,13 @@
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A211" s="7">
+      <c r="A211" s="10">
         <v>579</v>
       </c>
-      <c r="E211" s="2" t="s">
+      <c r="E211" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F211" s="2" t="s">
+      <c r="F211" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H211" s="2">
@@ -6109,13 +6127,13 @@
       </c>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A212" s="7">
+      <c r="A212" s="10">
         <v>580</v>
       </c>
-      <c r="E212" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F212" s="2" t="s">
+      <c r="E212" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F212" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H212" s="2">
@@ -6130,13 +6148,13 @@
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A213" s="7">
+      <c r="A213" s="10">
         <v>581</v>
       </c>
-      <c r="E213" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F213" s="2" t="s">
+      <c r="E213" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F213" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H213" s="2">
@@ -6151,13 +6169,13 @@
       </c>
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A214" s="7">
+      <c r="A214" s="10">
         <v>583</v>
       </c>
-      <c r="E214" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F214" s="2" t="s">
+      <c r="E214" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F214" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H214" s="2">
@@ -6172,13 +6190,13 @@
       </c>
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A215" s="7">
+      <c r="A215" s="10">
         <v>585</v>
       </c>
-      <c r="E215" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F215" s="2" t="s">
+      <c r="E215" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F215" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H215" s="2">
@@ -6193,13 +6211,13 @@
       </c>
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A216" s="7">
+      <c r="A216" s="10">
         <v>586</v>
       </c>
-      <c r="E216" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F216" s="2" t="s">
+      <c r="E216" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F216" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H216" s="2">
@@ -6214,13 +6232,13 @@
       </c>
     </row>
     <row r="217" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A217" s="7">
+      <c r="A217" s="10">
         <v>589</v>
       </c>
-      <c r="E217" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F217" s="2" t="s">
+      <c r="E217" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F217" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H217" s="2">
@@ -6235,13 +6253,13 @@
       </c>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A218" s="7">
+      <c r="A218" s="10">
         <v>590</v>
       </c>
-      <c r="E218" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F218" s="2" t="s">
+      <c r="E218" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F218" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H218" s="2">
@@ -6256,13 +6274,13 @@
       </c>
     </row>
     <row r="219" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A219" s="7">
+      <c r="A219" s="10">
         <v>591</v>
       </c>
-      <c r="E219" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F219" s="2" t="s">
+      <c r="E219" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F219" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H219" s="2">

</xml_diff>